<commit_message>
feat: add Vietnamese translation Excel files and update analysis cache data
</commit_message>
<xml_diff>
--- a/script_excel/sakumoyu-0054-kuro_002.xlsx
+++ b/script_excel/sakumoyu-0054-kuro_002.xlsx
@@ -7571,7 +7571,11 @@
         </is>
       </c>
       <c r="D327" t="inlineStr"/>
-      <c r="E327" t="inlineStr"/>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>Không hiểu sao khoé miệng tôi lại khẽ nhếch lên mỉm cười và nói— dẫu chính bản thân tôi cũng tự hỏi liệu đây có phải là chuyện nên nói vào lúc này hay không.</t>
+        </is>
+      </c>
       <c r="F327" t="inlineStr"/>
       <c r="G327" t="inlineStr"/>
     </row>
@@ -7592,7 +7596,11 @@
         </is>
       </c>
       <c r="D328" t="inlineStr"/>
-      <c r="E328" t="inlineStr"/>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>Có một hãng sản xuất loa và thiết bị âm thanh ấy.</t>
+        </is>
+      </c>
       <c r="F328" t="inlineStr"/>
       <c r="G328" t="inlineStr"/>
     </row>
@@ -7613,7 +7621,11 @@
         </is>
       </c>
       <c r="D329" t="inlineStr"/>
-      <c r="E329" t="inlineStr"/>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>...Hãng sản xuất sao?</t>
+        </is>
+      </c>
       <c r="F329" t="inlineStr"/>
       <c r="G329" t="inlineStr"/>
     </row>
@@ -7634,7 +7646,11 @@
         </is>
       </c>
       <c r="D330" t="inlineStr"/>
-      <c r="E330" t="inlineStr"/>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>...Ừm.</t>
+        </is>
+      </c>
       <c r="F330" t="inlineStr"/>
       <c r="G330" t="inlineStr"/>
     </row>
@@ -7655,7 +7671,11 @@
         </is>
       </c>
       <c r="D331" t="inlineStr"/>
-      <c r="E331" t="inlineStr"/>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>Thì cái đó đó. Có một logo rất nổi tiếng vẽ hình chú cún con ngồi trước một chiếc máy hát cổ và khẽ nghiêng đầu ấy.</t>
+        </is>
+      </c>
       <c r="F331" t="inlineStr"/>
       <c r="G331" t="inlineStr"/>
     </row>
@@ -7676,7 +7696,11 @@
         </is>
       </c>
       <c r="D332" t="inlineStr"/>
-      <c r="E332" t="inlineStr"/>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>Ừm. Đúng thế thật.</t>
+        </is>
+      </c>
       <c r="F332" t="inlineStr"/>
       <c r="G332" t="inlineStr"/>
     </row>
@@ -7693,7 +7717,11 @@
         </is>
       </c>
       <c r="D333" t="inlineStr"/>
-      <c r="E333" t="inlineStr"/>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>"Tớ từng thấy rồi." Cô gái gật đầu.</t>
+        </is>
+      </c>
       <c r="F333" t="inlineStr"/>
       <c r="G333" t="inlineStr"/>
     </row>
@@ -7714,7 +7742,11 @@
         </is>
       </c>
       <c r="D334" t="inlineStr"/>
-      <c r="E334" t="inlineStr"/>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>Từ chiếc máy hát đó phát ra giọng nói của người chủ đã khuất của chú cún... Chú cún cứ ngồi đó mãi không rời, nghển cổ nhìn vào chiếc máy đang phát ra giọng nói của người chủ mà nó yêu quý nhất—</t>
+        </is>
+      </c>
       <c r="F334" t="inlineStr"/>
       <c r="G334" t="inlineStr"/>
     </row>
@@ -7731,7 +7763,11 @@
         </is>
       </c>
       <c r="D335" t="inlineStr"/>
-      <c r="E335" t="inlineStr"/>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>Bức ảnh chụp lại khoảnh khắc tưởng nhớ chú cún ấy đã trở thành biểu tượng của công ty.</t>
+        </is>
+      </c>
       <c r="F335" t="inlineStr"/>
       <c r="G335" t="inlineStr"/>
     </row>
@@ -7748,7 +7784,11 @@
         </is>
       </c>
       <c r="D336" t="inlineStr"/>
-      <c r="E336" t="inlineStr"/>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>Có một giai thoại, hay nói đúng hơn là một "tin đồn" như vậy đấy...</t>
+        </is>
+      </c>
       <c r="F336" t="inlineStr"/>
       <c r="G336" t="inlineStr"/>
     </row>
@@ -7769,7 +7809,11 @@
         </is>
       </c>
       <c r="D337" t="inlineStr"/>
-      <c r="E337" t="inlineStr"/>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>Chỉ là tớ cảm giác cậu trông rất giống chú cún con đó...</t>
+        </is>
+      </c>
       <c r="F337" t="inlineStr"/>
       <c r="G337" t="inlineStr"/>
     </row>
@@ -7790,7 +7834,11 @@
         </is>
       </c>
       <c r="D338" t="inlineStr"/>
-      <c r="E338" t="inlineStr"/>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
       <c r="F338" t="inlineStr"/>
       <c r="G338" t="inlineStr"/>
     </row>
@@ -7807,7 +7855,11 @@
         </is>
       </c>
       <c r="D339" t="inlineStr"/>
-      <c r="E339" t="inlineStr"/>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>Cô gái chớp chớp đôi mắt to tròn.</t>
+        </is>
+      </c>
       <c r="F339" t="inlineStr"/>
       <c r="G339" t="inlineStr"/>
     </row>
@@ -7828,7 +7880,11 @@
         </is>
       </c>
       <c r="D340" t="inlineStr"/>
-      <c r="E340" t="inlineStr"/>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>Chú cún con đó... liệu có gặp lại được người chủ yêu quý của mình không?</t>
+        </is>
+      </c>
       <c r="F340" t="inlineStr"/>
       <c r="G340" t="inlineStr"/>
     </row>
@@ -7849,7 +7905,11 @@
         </is>
       </c>
       <c r="D341" t="inlineStr"/>
-      <c r="E341" t="inlineStr"/>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>...Đời nào chứ.</t>
+        </is>
+      </c>
       <c r="F341" t="inlineStr"/>
       <c r="G341" t="inlineStr"/>
     </row>
@@ -7866,7 +7926,11 @@
         </is>
       </c>
       <c r="D342" t="inlineStr"/>
-      <c r="E342" t="inlineStr"/>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>Tôi lắc đầu.</t>
+        </is>
+      </c>
       <c r="F342" t="inlineStr"/>
       <c r="G342" t="inlineStr"/>
     </row>
@@ -7887,7 +7951,11 @@
         </is>
       </c>
       <c r="D343" t="inlineStr"/>
-      <c r="E343" t="inlineStr"/>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>...Kẻ còn sống không bao giờ có thể gặp lại người đã khuất. Thế nên—</t>
+        </is>
+      </c>
       <c r="F343" t="inlineStr"/>
       <c r="G343" t="inlineStr"/>
     </row>
@@ -7904,7 +7972,11 @@
         </is>
       </c>
       <c r="D344" t="inlineStr"/>
-      <c r="E344" t="inlineStr"/>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>—Chắc chắn hai người họ đã không thể gặp lại nhau.</t>
+        </is>
+      </c>
       <c r="F344" t="inlineStr"/>
       <c r="G344" t="inlineStr"/>
     </row>
@@ -7925,7 +7997,11 @@
         </is>
       </c>
       <c r="D345" t="inlineStr"/>
-      <c r="E345" t="inlineStr"/>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>Đúng vậy nhỉ...</t>
+        </is>
+      </c>
       <c r="F345" t="inlineStr"/>
       <c r="G345" t="inlineStr"/>
     </row>
@@ -7942,7 +8018,11 @@
         </is>
       </c>
       <c r="D346" t="inlineStr"/>
-      <c r="E346" t="inlineStr"/>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>Thay vì gật đầu, cô gái khẽ nghiêng đầu.</t>
+        </is>
+      </c>
       <c r="F346" t="inlineStr"/>
       <c r="G346" t="inlineStr"/>
     </row>
@@ -7959,7 +8039,11 @@
         </is>
       </c>
       <c r="D347" t="inlineStr"/>
-      <c r="E347" t="inlineStr"/>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>...Giống hệt chú cún con kia.</t>
+        </is>
+      </c>
       <c r="F347" t="inlineStr"/>
       <c r="G347" t="inlineStr"/>
     </row>
@@ -7976,7 +8060,11 @@
         </is>
       </c>
       <c r="D348" t="inlineStr"/>
-      <c r="E348" t="inlineStr"/>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>Có điều, hành động ấy không hướng về chiếc máy hát trước mặt, mà là hướng về kẻ vừa đột ngột xuất hiện như tôi.</t>
+        </is>
+      </c>
       <c r="F348" t="inlineStr"/>
       <c r="G348" t="inlineStr"/>
     </row>
@@ -7997,7 +8085,11 @@
         </is>
       </c>
       <c r="D349" t="inlineStr"/>
-      <c r="E349" t="inlineStr"/>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>Cậu là...</t>
+        </is>
+      </c>
       <c r="F349" t="inlineStr"/>
       <c r="G349" t="inlineStr"/>
     </row>
@@ -8014,7 +8106,11 @@
         </is>
       </c>
       <c r="D350" t="inlineStr"/>
-      <c r="E350" t="inlineStr"/>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>"Ai vậy?"</t>
+        </is>
+      </c>
       <c r="F350" t="inlineStr"/>
       <c r="G350" t="inlineStr"/>
     </row>
@@ -8031,7 +8127,11 @@
         </is>
       </c>
       <c r="D351" t="inlineStr"/>
-      <c r="E351" t="inlineStr"/>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>Tôi cứ ngỡ cô ấy sẽ hỏi như vậy, thế nhưng—</t>
+        </is>
+      </c>
       <c r="F351" t="inlineStr"/>
       <c r="G351" t="inlineStr"/>
     </row>
@@ -8052,7 +8152,11 @@
         </is>
       </c>
       <c r="D352" t="inlineStr"/>
-      <c r="E352" t="inlineStr"/>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>Taiga.</t>
+        </is>
+      </c>
       <c r="F352" t="inlineStr"/>
       <c r="G352" t="inlineStr"/>
     </row>
@@ -8073,7 +8177,11 @@
         </is>
       </c>
       <c r="D353" t="inlineStr"/>
-      <c r="E353" t="inlineStr"/>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>Hả?</t>
+        </is>
+      </c>
       <c r="F353" t="inlineStr"/>
       <c r="G353" t="inlineStr"/>
     </row>
@@ -8094,7 +8202,11 @@
         </is>
       </c>
       <c r="D354" t="inlineStr"/>
-      <c r="E354" t="inlineStr"/>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>Kanade, Taiga...</t>
+        </is>
+      </c>
       <c r="F354" t="inlineStr"/>
       <c r="G354" t="inlineStr"/>
     </row>
@@ -8111,7 +8223,11 @@
         </is>
       </c>
       <c r="D355" t="inlineStr"/>
-      <c r="E355" t="inlineStr"/>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>"Đúng vậy không?" Cô gái mỉm cười nhẹ nhàng và nghiêng đầu hỏi.</t>
+        </is>
+      </c>
       <c r="F355" t="inlineStr"/>
       <c r="G355" t="inlineStr"/>
     </row>
@@ -8132,7 +8248,11 @@
         </is>
       </c>
       <c r="D356" t="inlineStr"/>
-      <c r="E356" t="inlineStr"/>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>Sao cậu lại biết tên tớ?</t>
+        </is>
+      </c>
       <c r="F356" t="inlineStr"/>
       <c r="G356" t="inlineStr"/>
     </row>
@@ -8153,7 +8273,11 @@
         </is>
       </c>
       <c r="D357" t="inlineStr"/>
-      <c r="E357" t="inlineStr"/>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>Tớ biết chứ.</t>
+        </is>
+      </c>
       <c r="F357" t="inlineStr"/>
       <c r="G357" t="inlineStr"/>
     </row>
@@ -8170,7 +8294,11 @@
         </is>
       </c>
       <c r="D358" t="inlineStr"/>
-      <c r="E358" t="inlineStr"/>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>Ngay lúc ấy, khúc ca phát ra từ máy hát cũng vừa kết thúc.</t>
+        </is>
+      </c>
       <c r="F358" t="inlineStr"/>
       <c r="G358" t="inlineStr"/>
     </row>
@@ -8191,7 +8319,11 @@
         </is>
       </c>
       <c r="D359" t="inlineStr"/>
-      <c r="E359" t="inlineStr"/>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>Chú cún tin tưởng đợi chủ nhân trở về có lẽ đã mãi mãi không thể gặp lại người nó yêu quý... Nhưng tớ thì khác, tớ đã gặp được cậu rồi này—</t>
+        </is>
+      </c>
       <c r="F359" t="inlineStr"/>
       <c r="G359" t="inlineStr"/>
     </row>
@@ -8208,7 +8340,11 @@
         </is>
       </c>
       <c r="D360" t="inlineStr"/>
-      <c r="E360" t="inlineStr"/>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>Cô gái nói.</t>
+        </is>
+      </c>
       <c r="F360" t="inlineStr"/>
       <c r="G360" t="inlineStr"/>
     </row>
@@ -8229,7 +8365,11 @@
         </is>
       </c>
       <c r="D361" t="inlineStr"/>
-      <c r="E361" t="inlineStr"/>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>Khoảnh khắc được gặp cậu trong "Dạ" thế này, tớ đã luôn chờ đợi từ rất lâu về trước—</t>
+        </is>
+      </c>
       <c r="F361" t="inlineStr"/>
       <c r="G361" t="inlineStr"/>
     </row>
@@ -8250,7 +8390,11 @@
         </is>
       </c>
       <c r="D362" t="inlineStr"/>
-      <c r="E362" t="inlineStr"/>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>Tớ đã chờ đợi cậu từ rất lâu, rất lâu trước cả khi cậu được sinh ra trên thế giới này đấy.</t>
+        </is>
+      </c>
       <c r="F362" t="inlineStr"/>
       <c r="G362" t="inlineStr"/>
     </row>

</xml_diff>